<commit_message>
test 78 per validazione
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\stefano\src\it-fse-accreditamento\GATEWAY\S1#111#DIGITALMINDSSRLXX\digitalminds\XilemaFSE\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{830CAFB3-7A5C-4CF0-97D0-D3A24F789CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39A634BD-D59C-44EC-8A6B-4EF126827C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2250" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="oXWj5iU3LtnvLpdhFqszSz/X91q3fG5U5zC5TJKtiGw="/>
     </ext>
   </extLst>
 </workbook>
@@ -80,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="221">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -915,6 +912,33 @@
   <si>
     <t>Al salvataggio del referto viene verificata la validità del codice fiscale, avvisando l'utente e permettendo una correzione per tempo. Qualora si dovesse incappare in questo errore lo stesso, viene mostrato il messaggio di errore a video e l'utente è invitato a controllare il codice fiscale per correggerlo. A quel punto può rigenerare il referto e ripetere la procedura.</t>
   </si>
+  <si>
+    <t>2026-03-20T12:08:49.039Z</t>
+  </si>
+  <si>
+    <t>fbf6c52ddfb0d6105fc1b02f7d69104b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.4.1.1.700261e95ee36ad94b40e3adab904b398048724a8c8c5396e2e40980a0365fcd.114ebc235c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>[ERRORE-11| L'elemento ClinicalDocument/recordTarget/patientRole/addr DEVE riportare i suoi sotto-elementi 'country', 'city' e 'streetAddressLine'.   ]</t>
+  </si>
+  <si>
+    <t>Questa problematica viene prevenuta da un controllo prima della generazione del referto: tutti i dati del paziente devono essere presenti e correttamente compilati. La gestione dell'errore è quindi di tipo preventivo.</t>
+  </si>
+  <si>
+    <t>L'applicazione non gestisce le immagini DICOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> "effectivetime/low" ha sempre un valore di default, se non è presente la data perché non è disponbile  allora è presente il valore @nullFlavor = “UNK”.</t>
+  </si>
+  <si>
+    <t>La storia clinica non è gestita</t>
+  </si>
+  <si>
+    <t>Le allergie non vengono gestite</t>
+  </si>
 </sst>
 </file>
 
@@ -923,11 +947,18 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1061,7 +1092,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -1370,174 +1401,221 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal 2" xfId="1" xr:uid="{565105C8-FFD6-432C-8B2E-BD1D172FCD26}"/>
+    <cellStyle name="Normal 2 2" xfId="2" xr:uid="{816B634F-18CD-48D3-B461-04313602D5C7}"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
@@ -2972,6 +3050,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W558"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3314,7 +3393,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:23" ht="145.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="31">
         <v>32</v>
       </c>
@@ -3410,7 +3489,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="145.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:23" ht="145.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="31">
         <v>40</v>
       </c>
@@ -3504,7 +3583,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="87.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:23" ht="87.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="31">
         <v>48</v>
       </c>
@@ -3602,7 +3681,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:23" ht="116.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="31">
         <v>78</v>
       </c>
@@ -3618,20 +3697,44 @@
       <c r="E17" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="33"/>
+      <c r="F17" s="32">
+        <v>46101</v>
+      </c>
+      <c r="G17" s="32" t="s">
+        <v>212</v>
+      </c>
+      <c r="H17" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>214</v>
+      </c>
+      <c r="J17" s="33" t="s">
+        <v>61</v>
+      </c>
       <c r="K17" s="33"/>
       <c r="L17" s="33"/>
-      <c r="M17" s="33"/>
-      <c r="N17" s="33"/>
-      <c r="O17" s="33"/>
-      <c r="P17" s="33"/>
-      <c r="Q17" s="33"/>
-      <c r="R17" s="33"/>
-      <c r="S17" s="33"/>
+      <c r="M17" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="N17" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="O17" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="P17" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q17" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="R17" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="S17" s="33" t="s">
+        <v>216</v>
+      </c>
       <c r="T17" s="33"/>
       <c r="U17" s="34"/>
       <c r="V17" s="35"/>
@@ -3659,8 +3762,12 @@
       <c r="G18" s="32"/>
       <c r="H18" s="32"/>
       <c r="I18" s="37"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
+      <c r="J18" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K18" s="33" t="s">
+        <v>151</v>
+      </c>
       <c r="L18" s="33"/>
       <c r="M18" s="33"/>
       <c r="N18" s="33"/>
@@ -3696,8 +3803,12 @@
       <c r="G19" s="32"/>
       <c r="H19" s="32"/>
       <c r="I19" s="37"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="33"/>
+      <c r="J19" s="63" t="s">
+        <v>193</v>
+      </c>
+      <c r="K19" s="63" t="s">
+        <v>154</v>
+      </c>
       <c r="L19" s="33"/>
       <c r="M19" s="33"/>
       <c r="N19" s="33"/>
@@ -3733,8 +3844,12 @@
       <c r="G20" s="32"/>
       <c r="H20" s="32"/>
       <c r="I20" s="37"/>
-      <c r="J20" s="33"/>
-      <c r="K20" s="33"/>
+      <c r="J20" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K20" s="63" t="s">
+        <v>154</v>
+      </c>
       <c r="L20" s="33"/>
       <c r="M20" s="33"/>
       <c r="N20" s="33"/>
@@ -3770,8 +3885,12 @@
       <c r="G21" s="32"/>
       <c r="H21" s="32"/>
       <c r="I21" s="37"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
+      <c r="J21" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K21" s="63" t="s">
+        <v>154</v>
+      </c>
       <c r="L21" s="33"/>
       <c r="M21" s="33"/>
       <c r="N21" s="33"/>
@@ -3807,8 +3926,12 @@
       <c r="G22" s="32"/>
       <c r="H22" s="32"/>
       <c r="I22" s="37"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
+      <c r="J22" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K22" s="63" t="s">
+        <v>154</v>
+      </c>
       <c r="L22" s="33"/>
       <c r="M22" s="33"/>
       <c r="N22" s="33"/>
@@ -3881,8 +4004,12 @@
       <c r="G24" s="32"/>
       <c r="H24" s="32"/>
       <c r="I24" s="37"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="33"/>
+      <c r="J24" s="33" t="s">
+        <v>193</v>
+      </c>
+      <c r="K24" s="63" t="s">
+        <v>154</v>
+      </c>
       <c r="L24" s="33"/>
       <c r="M24" s="33"/>
       <c r="N24" s="33"/>
@@ -3918,9 +4045,15 @@
       <c r="G25" s="32"/>
       <c r="H25" s="32"/>
       <c r="I25" s="37"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="33"/>
-      <c r="L25" s="33"/>
+      <c r="J25" s="64" t="s">
+        <v>193</v>
+      </c>
+      <c r="K25" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="L25" s="64" t="s">
+        <v>217</v>
+      </c>
       <c r="M25" s="33"/>
       <c r="N25" s="33"/>
       <c r="O25" s="33"/>
@@ -3955,9 +4088,15 @@
       <c r="G26" s="32"/>
       <c r="H26" s="32"/>
       <c r="I26" s="37"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
+      <c r="J26" s="65" t="s">
+        <v>193</v>
+      </c>
+      <c r="K26" s="65" t="s">
+        <v>156</v>
+      </c>
+      <c r="L26" s="65" t="s">
+        <v>218</v>
+      </c>
       <c r="M26" s="33"/>
       <c r="N26" s="33"/>
       <c r="O26" s="33"/>
@@ -3992,9 +4131,15 @@
       <c r="G27" s="32"/>
       <c r="H27" s="32"/>
       <c r="I27" s="37"/>
-      <c r="J27" s="33"/>
-      <c r="K27" s="33"/>
-      <c r="L27" s="33"/>
+      <c r="J27" s="66" t="s">
+        <v>193</v>
+      </c>
+      <c r="K27" s="66" t="s">
+        <v>156</v>
+      </c>
+      <c r="L27" s="66" t="s">
+        <v>219</v>
+      </c>
       <c r="M27" s="33"/>
       <c r="N27" s="33"/>
       <c r="O27" s="33"/>
@@ -4029,9 +4174,15 @@
       <c r="G28" s="32"/>
       <c r="H28" s="32"/>
       <c r="I28" s="37"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="33"/>
+      <c r="J28" s="66" t="s">
+        <v>193</v>
+      </c>
+      <c r="K28" s="66" t="s">
+        <v>156</v>
+      </c>
+      <c r="L28" s="66" t="s">
+        <v>218</v>
+      </c>
       <c r="M28" s="33"/>
       <c r="N28" s="33"/>
       <c r="O28" s="33"/>
@@ -4066,9 +4217,15 @@
       <c r="G29" s="32"/>
       <c r="H29" s="32"/>
       <c r="I29" s="37"/>
-      <c r="J29" s="33"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
+      <c r="J29" s="67" t="s">
+        <v>193</v>
+      </c>
+      <c r="K29" s="67" t="s">
+        <v>156</v>
+      </c>
+      <c r="L29" s="67" t="s">
+        <v>220</v>
+      </c>
       <c r="M29" s="33"/>
       <c r="N29" s="33"/>
       <c r="O29" s="33"/>
@@ -4103,8 +4260,12 @@
       <c r="G30" s="32"/>
       <c r="H30" s="32"/>
       <c r="I30" s="37"/>
-      <c r="J30" s="33"/>
-      <c r="K30" s="33"/>
+      <c r="J30" s="68" t="s">
+        <v>193</v>
+      </c>
+      <c r="K30" s="68" t="s">
+        <v>154</v>
+      </c>
       <c r="L30" s="33"/>
       <c r="M30" s="33"/>
       <c r="N30" s="33"/>
@@ -4140,8 +4301,12 @@
       <c r="G31" s="32"/>
       <c r="H31" s="32"/>
       <c r="I31" s="37"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="33"/>
+      <c r="J31" s="69" t="s">
+        <v>193</v>
+      </c>
+      <c r="K31" s="69" t="s">
+        <v>154</v>
+      </c>
       <c r="L31" s="33"/>
       <c r="M31" s="33"/>
       <c r="N31" s="33"/>
@@ -4157,7 +4322,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="31">
         <v>152</v>
       </c>
@@ -4194,7 +4359,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="31">
         <v>154</v>
       </c>
@@ -4231,7 +4396,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="31">
         <v>155</v>
       </c>
@@ -4268,7 +4433,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="31">
         <v>156</v>
       </c>
@@ -4305,7 +4470,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="36" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="31">
         <v>159</v>
       </c>
@@ -4342,7 +4507,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="31">
         <v>160</v>
       </c>
@@ -4379,7 +4544,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="31">
         <v>161</v>
       </c>
@@ -4416,7 +4581,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="31">
         <v>162</v>
       </c>
@@ -4453,7 +4618,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="31">
         <v>163</v>
       </c>
@@ -4490,7 +4655,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="31">
         <v>164</v>
       </c>
@@ -4527,7 +4692,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="31">
         <v>165</v>
       </c>
@@ -4564,7 +4729,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="31">
         <v>166</v>
       </c>
@@ -4601,7 +4766,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="31">
         <v>167</v>
       </c>
@@ -4638,7 +4803,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="31">
         <v>168</v>
       </c>
@@ -4675,7 +4840,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="31">
         <v>169</v>
       </c>
@@ -4712,7 +4877,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:23" ht="131" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="31">
         <v>448</v>
       </c>
@@ -4749,7 +4914,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="131" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:23" ht="131" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="31">
         <v>449</v>
       </c>
@@ -4786,7 +4951,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="31">
         <v>461</v>
       </c>
@@ -4860,7 +5025,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="31">
         <v>468</v>
       </c>
@@ -5008,7 +5173,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="102" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:23" ht="102" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="31">
         <v>475</v>
       </c>
@@ -8017,7 +8182,13 @@
       <c r="W558" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A9:W55" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A9:W55" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="RAD"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="7">
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:B2"/>
@@ -8027,7 +8198,7 @@
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
   </mergeCells>
-  <phoneticPr fontId="15" type="noConversion"/>
+  <phoneticPr fontId="16" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
   <legacyDrawing r:id="rId1"/>
@@ -8038,7 +8209,7 @@
           <x14:formula1>
             <xm:f>Sheet1!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J11:J55 M11:N55 P10:R55</xm:sqref>
+          <xm:sqref>P10:R55 M11:N55 J11:J55</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{70793024-27E9-4E6A-BACD-083AB683BC38}">
           <x14:formula1>
@@ -10335,6 +10506,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -10598,28 +10790,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10638,31 +10834,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>

<commit_message>
test 471 secondo tentativo
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\darcast\src\git-hub\it-fse-accreditamento\GATEWAY\S1#111#DIGITALMINDSSRLXX\digitalminds\XilemaFSE\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F30AC82-67C2-47D9-95E2-39C7B53FE613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFFBCF3-A71C-4D95-BA74-B6EC0DE73031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -806,16 +806,16 @@
     <t xml:space="preserve">Prima dell'invio del referto viene effettuata la validazione dei dati del referto,  permettendo una correzione prima dell'invio del referto. </t>
   </si>
   <si>
-    <t>2026-03-26T15:05:44.710Z</t>
-  </si>
-  <si>
-    <t>5f240523db09769b2e1a112c74ac96ce</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.4.1.1.0fb1500ecf47cec8ffb9c5312b85ea027118c7e7e62869e4b2a17eaa97bcfe7f.7ae4522e1f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Il software non gestisce la storia clinica e le allegie</t>
+  </si>
+  <si>
+    <t>3d0ebf26ce68b2ccd5f4dad228406959</t>
+  </si>
+  <si>
+    <t>2026-03-31T15:02:42.270Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.4.1.1.3b6a4c22308c452911b141d984dc5c2a72ca611c6b68257cfb546a84def6795d.812c5223d2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -4158,16 +4158,16 @@
         <v>97</v>
       </c>
       <c r="F30" s="32">
-        <v>46107</v>
+        <v>46112</v>
       </c>
       <c r="G30" s="32" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="H30" s="32" t="s">
         <v>184</v>
       </c>
       <c r="I30" s="37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J30" s="33" t="s">
         <v>59</v>
@@ -4215,7 +4215,7 @@
         <v>113</v>
       </c>
       <c r="L31" s="33" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="M31" s="33"/>
       <c r="N31" s="33"/>
@@ -9562,12 +9562,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9835,21 +9838,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9874,18 +9883,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Correzione data esame eseguito
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\darcast\src\git-hub\it-fse-accreditamento\GATEWAY\S1#111#DIGITALMINDSSRLXX\digitalminds\XilemaFSE\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFFBCF3-A71C-4D95-BA74-B6EC0DE73031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289E76B9-9B66-4CAA-BC46-BB268F85A942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -809,13 +809,13 @@
     <t>Il software non gestisce la storia clinica e le allegie</t>
   </si>
   <si>
-    <t>3d0ebf26ce68b2ccd5f4dad228406959</t>
-  </si>
-  <si>
-    <t>2026-03-31T15:02:42.270Z</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.4.1.1.3b6a4c22308c452911b141d984dc5c2a72ca611c6b68257cfb546a84def6795d.812c5223d2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-02T09:12:06.717Z</t>
+  </si>
+  <si>
+    <t>5a13db8201200b23dd3f887ea81699c9</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.4.1.1.87bd96acfd2e31503b6694011a6be68881222b79145591c9be3b76d3b7029194.f8d72f1848^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -3374,7 +3374,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:23" s="50" customFormat="1" ht="225.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" s="50" customFormat="1" ht="210.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="41">
         <v>76</v>
       </c>
@@ -4158,13 +4158,13 @@
         <v>97</v>
       </c>
       <c r="F30" s="32">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="G30" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="H30" s="32" t="s">
         <v>185</v>
-      </c>
-      <c r="H30" s="32" t="s">
-        <v>184</v>
       </c>
       <c r="I30" s="37" t="s">
         <v>186</v>
@@ -9562,18 +9562,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -9837,6 +9825,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9847,23 +9847,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9882,6 +9865,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Rimosso low su effective date di esame eseguito
</commit_message>
<xml_diff>
--- a/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/S1#111#DIGITALMINDSSRLXX/digitalminds/XilemaFSE/1.0.0/report-checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\darcast\src\git-hub\it-fse-accreditamento\GATEWAY\S1#111#DIGITALMINDSSRLXX\digitalminds\XilemaFSE\1.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289E76B9-9B66-4CAA-BC46-BB268F85A942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{222EB675-B280-4A54-B5AC-031F4DC61D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -809,13 +809,13 @@
     <t>Il software non gestisce la storia clinica e le allegie</t>
   </si>
   <si>
-    <t>2026-04-02T09:12:06.717Z</t>
-  </si>
-  <si>
-    <t>5a13db8201200b23dd3f887ea81699c9</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.4.1.1.87bd96acfd2e31503b6694011a6be68881222b79145591c9be3b76d3b7029194.f8d72f1848^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-04-07T18:32:32.899Z</t>
+  </si>
+  <si>
+    <t>bdb4277fcb95222533a1fdc6b1c47c6d</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.4.1.1.b200ff8f52bde9816d554c83cbad43338291415dd2602c189424605934866de6.0b1639d23a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -4158,7 +4158,7 @@
         <v>97</v>
       </c>
       <c r="F30" s="32">
-        <v>46114</v>
+        <v>46119</v>
       </c>
       <c r="G30" s="32" t="s">
         <v>184</v>
@@ -9562,6 +9562,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -9825,18 +9837,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -9847,6 +9847,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9865,23 +9882,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>

</xml_diff>